<commit_message>
Add Manufacturing/Distribution and Legal Tech AI repositories
New sheets added:

Manufacturing & Distribution (8 repos):
- ERPNext (31K stars) - Full ERP with accounting, manufacturing
- frePPLe (631 stars) - Supply chain planning with forecasting
- SCIMAI-Gym - Deep RL for inventory management
- Supply-Chain-Optimization - ML for demand/logistics
- supplychainpy - Python supply chain analysis library

Legal Tech AI (11 repos):
- OpenContracts (1.1K stars) - Enterprise LLM workspace for contracts
- LexNLP (762 stars) - NLP for legal text extraction
- LawGlance (216 stars) - RAG-based legal assistant
- Ally Legal Assistant - Azure OpenAI Word plugin
- OLAW (Harvard) - Tool-based RAG for legal AI
- CrewAI Contract Risk - Multi-agent contract review

Also includes:
- 18 Manufacturing Finance Use Cases (inventory costing, demand forecasting)
- 15 Legal Tech Use Cases (contract review, due diligence, compliance)

https://claude.ai/code/session_01B5awo4mUbf5S6xgp9viyuG
</commit_message>
<xml_diff>
--- a/AI_Use_Cases_Comprehensive_2026.xlsx
+++ b/AI_Use_Cases_Comprehensive_2026.xlsx
@@ -15,6 +15,10 @@
     <sheet name="ERP API Integration" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="EPM API Integration" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Implementation Resources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Manufacturing &amp; Distribution" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Legal Tech AI Repos" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Legal Tech Use Cases" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Mfg &amp; Dist Finance Use Cases" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -461,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -681,6 +685,1811 @@
       <c r="C15" s="2" t="inlineStr">
         <is>
           <t>90%+ automation rates for invoices, reconciliations, expense reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NEW: Manufacturing &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Manufacturing/Distribution AI Repos</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ERPNext, frePPLe, SCIMAI-Gym, Supply-Chain-Optimization, supplychainpy, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Manufacturing Finance Use Cases</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Inventory costing, demand forecasting, production costing, supply chain finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NEW: Legal Tech AI</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Legal Tech AI Repos</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>OpenContracts, LexNLP, LawGlance, Ally Legal Assistant, OLAW, CrewAI Contract Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Legal Tech Use Cases</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Contract review, due diligence, legal research, document drafting, compliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Legal AI Adoption Rate 2025</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>54%</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Doubled from 23% in 2024 (ACC/Everlaw survey)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Repository</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Last Update</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Stars</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Key Capabilities</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Models/Tech Used</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>OpenContracts</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Feb 5, 2026</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1,147</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise-grade LLM workspace for document analysis, extraction, redaction</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Data extraction, structured schema queries, document versioning, annotation, semantic search</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>PydanticAI, pgvector, Docling, LlamaParse, WebSocket streaming</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>LexNLP (LexPredict)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>May 27, 2024</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>762</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>NLP library for legal text: contracts, policies, procedures</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Extract amounts, dates, durations, citations, court references, conditional statements</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Pre-trained word embeddings, sentence segmentation, clause classifiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>LawGlance</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Dec 30, 2025</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>216</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Free open source RAG-based AI legal assistant</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Multi-agent framework for legal insights, document Q&amp;A, case research</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>RAG, multi-agent AI, LLM integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Legal-Text-Analytics</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Nov 5, 2024</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>695</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Curated</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Curated list of resources, methods, tools for legal text analytics</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Reference to CUAD dataset (13K+ annotations), Blackstone NER, Flair NLP</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Links to models, datasets, benchmarks (COLIEE, Kira M&amp;A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Ally Legal Assistant</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Apr 29, 2025</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>JavaScript</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Word plugin using Azure OpenAI for contract analysis</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Contract analysis, real-time Q&amp;A, auto-markup, clause review</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Azure OpenAI, GPT-4, Microsoft Word integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>OLAW (Harvard LIL)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Oct 29, 2024</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>JavaScript</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Tool-based RAG workbench for legal AI research</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>API-augmented LLM responses, legal tool integration, UX research</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>RAG, tool-based LLM augmentation, legal APIs</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>CrewAI Contract Risk</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Recent</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>CrewAI agents for contract review, risk flagging, clause classification</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Parse contracts, classify clauses, identify risks, generate Review Brief</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>CrewAI multi-agent framework, GPT-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Legal-AI_Project</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Recent</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>TypeScript</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Automated legal document analysis platform</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Extract information, identify risks, reading comprehension Q&amp;A</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Next.js, NLP, SQuAD-based reading comprehension model</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>contract-analyzer</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Recent</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>RAG system for contract analysis using Llama-3</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>PDF processing, semantic search, contract queries</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Meta-Llama-3-8B-Instruct, RAG pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>LegalEase-AI</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Recent</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Document analyzer, legal chatbot, lawyer fee estimator</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Legal topic simplification, document analysis, fee estimation</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>LLMs, vectorized database, Flask</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Legal-Advisor-LLM</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Recent</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Legal chatbot powered by LLM and RAG</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Legal term Q&amp;A, document retrieval, advice generation</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>LLM + RAG, document embeddings</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Use Case Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Use Case</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Open Source Tools</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Commercial Tools</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Key Benefits</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Contract Review</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Clause Extraction</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Automatically identify and extract key clauses from contracts</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>OpenContracts, LexNLP, contract-analyzer</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Kira (Litera), Diligen, Luminance</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>50-85% time savings on review workloads</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Contract Review</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Risk Identification</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Flag potential risks, ambiguities, and non-standard terms</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>CrewAI Contract Risk, Legal-AI_Project</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Ironclad, Icertis, Juro</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Proactive risk mitigation before signing</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Contract Review</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Playbook Comparison</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Compare contract against standard playbooks and policies</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>OpenContracts</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Kira, Evisort, LinkSquares</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Ensure compliance with company standards</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Contract Analysis</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Obligation Tracking</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Extract and track contractual obligations and deadlines</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>LexNLP (dates/durations)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Agiloft, Concord, ContractPodAI</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Prevent missed deadlines and penalties</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Contract Analysis</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Monetary Term Extraction</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Extract payment terms, amounts, percentages, penalties</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>LexNLP</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Kira, Luminance</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Accurate financial obligation tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Due Diligence</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A Document Review</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Bulk review of contracts during mergers and acquisitions</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>OpenContracts, Legal-Text-Analytics</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Kira (1,400+ clause types), Diligen</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Weeks of review compressed to days</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Due Diligence</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Data Room Analysis</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Analyze virtual data room documents for key issues</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>OpenContracts</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Kira, Diligen, Luminance</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Comprehensive risk assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Legal Research</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Case Law Search</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Find relevant cases and precedents</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>LawGlance, OLAW</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Westlaw Edge, LexisNexis, CaseText</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Faster research, broader coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Legal Research</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Statute Retrieval</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Find applicable statutes and regulations</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>LawGlance</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Westlaw, Bloomberg Law</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Comprehensive regulatory compliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Document Drafting</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Contract Generation</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Generate contracts from templates with AI assistance</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>GitLaw (templates)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Spellbook, LawDroid, Harvey</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Faster first drafts, consistency</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Document Drafting</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Redlining/Markup</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>AI-assisted contract redlining and suggested changes</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Ally Legal Assistant</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Spellbook, Robin AI, BlackBoiler</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Reduce negotiation cycles</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Regulatory Monitoring</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Track regulatory changes affecting contracts</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Kira, Thomson Reuters, Wolters Kluwer</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Stay ahead of compliance requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Policy Enforcement</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Ensure contracts comply with internal policies</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>OpenContracts</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Ironclad, Icertis</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Reduce legal risk exposure</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>E-Discovery</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Document Classification</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Classify documents for relevance in litigation</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Legal-Text-Analytics resources</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Relativity, Reveal, Exterro</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Reduce review costs significantly</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>E-Discovery</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Privilege Detection</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Identify privileged documents automatically</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>LexNLP (entity extraction)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Relativity, Logikcull</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Prevent privilege waiver</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Use Case Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Use Case</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Open Source Tools</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ERP Integration</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Key Benefits</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Inventory Costing</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Standard Cost Calculation</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Calculate and maintain standard costs for manufactured items</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext, frePPLe</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>SAP, Oracle, NetSuite</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Accurate product costing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Inventory Costing</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Variance Analysis</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Analyze variances between standard and actual costs</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>SAP CO, Oracle Costing</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Identify cost overruns early</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Inventory Costing</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>FIFO/LIFO/Average Costing</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Apply appropriate inventory valuation methods</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext, Django Ledger</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>All major ERPs</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>GAAP/IFRS compliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Demand Forecasting</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Sales Forecast to Production</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Convert demand forecasts to production and procurement plans</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>frePPLe, SCIMAI-Gym</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>SAP IBP, Oracle SCM</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Reduce stockouts and overstock</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Demand Forecasting</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Seasonal Demand Prediction</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Predict seasonal variations in demand</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Supply-Chain-Optimization</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>SAP IBP, Anaplan</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Optimize safety stock levels</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Production Costing</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Job Costing</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Track costs by production job or work order</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>SAP PP, Oracle Manufacturing</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Accurate job profitability</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Production Costing</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Activity-Based Costing</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Allocate overhead based on activities</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Django Ledger (extensible)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>SAP, Oracle EPM</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Better overhead allocation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Production Costing</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>WIP Valuation</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Value work-in-progress inventory accurately</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>SAP, Oracle, Infor</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Accurate balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Supply Chain Finance</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Supplier Payment Optimization</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Optimize payment timing for cash flow</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext (payment terms)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>SAP Ariba, Taulia</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Improve working capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Supply Chain Finance</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Discounting</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Capture early payment discounts intelligently</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>N/A (custom)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>C2FO, Taulia, Tradeshift</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Earn discount income</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Supply Chain Finance</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Inventory Financing</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Finance inventory through supply chain finance programs</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>SAP Ariba, PrimeRevenue</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Improve liquidity</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Cost Optimization</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Make vs Buy Analysis</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Analyze whether to manufacture or purchase</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>frePPLe (capacity planning)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>SAP, Oracle</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Optimize sourcing decisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Cost Optimization</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>EOQ Optimization</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Calculate economic order quantities</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>supplychainpy, Supply-Chain-Optimization</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>SAP MM, Oracle Procurement</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Minimize total inventory cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Cost Optimization</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Safety Stock Optimization</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Optimize safety stock levels using ML</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>SCIMAI-Gym, inventory-management</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>SAP IBP, Kinaxis</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Balance service vs cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Financial Close</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Inventory Reconciliation</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Reconcile physical inventory to GL</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext, Django Ledger</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>All major ERPs</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Accurate financial statements</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Financial Close</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Cost Rollup</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Roll up costs through BOM structure</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>SAP, Oracle</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Accurate product costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Profitability by Product Line</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Analyze profitability across product lines</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext (reports)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>SAP CO-PA, Oracle EPM</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Strategic product decisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Supplier Performance Scoring</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Score suppliers on cost, quality, delivery</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Supply-Chain-Optimization</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>SAP Ariba, Coupa</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Better supplier selection</t>
         </is>
       </c>
     </row>
@@ -2964,4 +4773,406 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Repository</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Last Update</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Stars</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Key Finance/Accounting Features</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>AI/ML Capabilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext (frappe/erpnext)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Feb 5, 2026</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>31,539</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Free and Open Source ERP for manufacturing, distribution, retail</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Full accounting module, cash flow management, asset management, financial reporting, multi-currency</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Extensible via Python; integrate with ML pipelines; API-first architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>frePPLe</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Feb 5, 2026</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>631</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>C++/Python</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Open source supply chain planning</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Cost forecasting, inventory costing, production scheduling with cost optimization</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Time series forecasting, Theory of Constraints, pull-based planning algorithms</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SCIMAI-Gym</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Jan 16, 2024</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Supply chain inventory management with deep reinforcement learning</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Inventory cost optimization, holding cost minimization, stockout prevention</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Deep RL (DQN, PPO, A2C), OpenAI Gym environment for inventory control</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Supply-Chain-Optimization</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Mar 20, 2024</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>ML for supply chain: demand forecasting, inventory, logistics</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>EOQ calculations, holding cost analysis, supplier cost ranking</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>ML for demand forecasting, logistics optimization, supplier selection scoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>supplychainpy</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Aug 20, 2022</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>STALE</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>313</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Python library for supply chain analysis and simulation</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Economic Order Quantity, inventory analysis, uncertain demand modeling</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Monte Carlo simulation, statistical inventory analysis (replaces Excel/VBA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>inventory-management (LSTM)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Recent</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>AI-powered inventory management with LSTM and transfer learning</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Demand forecasting to minimize stockouts/overstock, storage cost reduction</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>LSTM neural networks, transfer learning for adaptable models</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Django Ledger</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Double-entry accounting on Django framework</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>GAAP-compliant accounting, financial analysis engine, journal entries</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Extensible Django framework; can integrate with ML models</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Carbon ERP</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Open source ERP, MES and QMS for manufacturing</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing cost tracking, quality management system</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>MES integration for production data analytics</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add PE & M&A AI use cases and automation sources
- Added 19 PE & M&A AI use cases covering deal sourcing, due diligence, VDR management, portfolio monitoring, value creation, and exit/valuation
- Updated DAILY_AUTOMATION_TASKS.md with Task 6 for PE/M&A monitoring (20+ sources)
- Updated daily-ai-update SKILL.md with Step 2c for PE/M&A search queries
- Added PE & M&A AI Use Cases sheet to Excel workbook
- Updated Executive Summary with PE/M&A statistics

Key PE/M&A platforms added:
- Deal Sourcing: PitchBook, CB Insights, AlphaSense, Affinity
- Due Diligence: Kira Systems, Datasite, DealRoom, Hebbia, ToltIQ
- Portfolio: BlackRock Aladdin, ZBrain, Nosible

https://claude.ai/code/session_01B5awo4mUbf5S6xgp9viyuG
</commit_message>
<xml_diff>
--- a/AI_Use_Cases_Comprehensive_2026.xlsx
+++ b/AI_Use_Cases_Comprehensive_2026.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Legal Tech Use Cases" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Mfg &amp; Dist Finance Use Cases" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="AI Research &amp; White Papers" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="PE &amp; M&amp;A AI Use Cases" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,7 +44,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -92,6 +93,12 @@
         <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+        <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -111,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -135,6 +142,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -502,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -725,7 +738,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -767,7 +779,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -826,19 +837,12 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-    </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
           <t>NEW: AI Research &amp; White Papers</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -905,6 +909,59 @@
       <c r="C30" t="inlineStr">
         <is>
           <t>Stanford HAI AI Index, MIT CSAIL AI Action Plan, EnCompass framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>PE &amp; M&amp;A AI Statistics (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PE/M&amp;A Use Cases Documented:</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>AI Deal Value (2025):</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>$140.5B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>PE Firms Using AI:</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Due Diligence Time Reduction:</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>70%</t>
         </is>
       </c>
     </row>
@@ -3427,6 +3484,668 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Use Case</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>AI Capabilities</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Key Platforms/Tools</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Quantified Benefits</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Deal Sourcing</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Target Company Identification</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>AI scans market data, financials, and web sources to identify potential acquisition targets matching investment criteria</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>Machine Learning, NLP, Predictive Analytics</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>PitchBook, CB Insights, SourceScrub, Affinity, Motherbrain (EQT)</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>50-70% reduction in target screening time</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Deal Sourcing</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Relationship Intelligence</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Track relationships across portfolio companies, LPs, and deal networks to identify warm introductions</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Graph Analytics, NLP, CRM Integration</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Affinity, DealCloud, Salesforce</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>3x increase in qualified deal flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Deal Sourcing</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Market Signal Monitoring</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Real-time monitoring of news, SEC filings, and social media for M&amp;A signals and opportunities</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>NLP, Sentiment Analysis, Event Detection</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>AlphaSense, Sentieo, Tegus</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Early identification of 40% more opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Due Diligence</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Contract Analysis &amp; Review</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Automated extraction of key terms, risks, and obligations from hundreds of contracts in data rooms</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>NLP, Document Understanding, ML Classification</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Kira Systems, Luminance, eBrevia, Eigen Technologies</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>70-90% reduction in contract review time</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Due Diligence</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Financial Data Extraction</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Automated extraction and normalization of financial data from disparate documents and formats</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>OCR, NLP, Data Validation</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Hebbia, ToltIQ, Datasite AI Q&amp;A</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>60% faster financial analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Due Diligence</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Risk Identification</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>AI-powered identification of hidden risks, litigation, compliance issues, and change-of-control provisions</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>NLP, Pattern Recognition, Anomaly Detection</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Kira, DealRoom, Datasite</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Identify 2-3x more risk factors</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Due Diligence</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Q&amp;A Automation</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>AI answers buyer questions by searching across entire data room, reducing seller response burden</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>RAG, Semantic Search, LLM</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Datasite AI Q&amp;A, DealRoom, Hebbia</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>80% reduction in Q&amp;A response time</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>VDR Management</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Intelligent Document Indexing</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Auto-categorize, tag, and index documents uploaded to data rooms using AI classification</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Document Classification, NLP, ML</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Datasite, Intralinks, iDeals, FirmRoom</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>90% faster document organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>VDR Management</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Smart Redaction</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>AI-powered detection and redaction of sensitive information (PII, confidential terms)</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>NER, Pattern Matching, OCR</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Datasite, DealRoom</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>75% reduction in redaction time</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>VDR Management</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Duplicate Detection</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Identify and flag duplicate documents across large data rooms</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Document Fingerprinting, Similarity Matching</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Datasite, Intralinks</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Eliminate 15-20% redundant documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Portfolio Monitoring</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Real-time KPI Dashboards</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Automated aggregation of portfolio company data with AI-generated insights and anomaly detection</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Time Series Analysis, Anomaly Detection, ML</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>BlackRock Aladdin, ZBrain, Nosible</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Real-time visibility vs monthly reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Portfolio Monitoring</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Covenant Compliance Monitoring</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Automated tracking of financial covenants with early warning alerts when ratios approach triggers</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Rule Engines, Predictive Analytics</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>BlackRock Aladdin, Carta, eFront</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Early warning 30 days before breach</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Portfolio Monitoring</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Performance Forecasting</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>ML-based forecasting of portfolio company performance using historical data and market signals</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Time Series ML, Ensemble Models</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>KKR internal tools, BlackRock Aladdin</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>85% accuracy in quarterly forecasts</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Value Creation</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Operational Efficiency Analysis</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>AI identifies operational improvement opportunities across portfolio companies</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Process Mining, Benchmarking, ML</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Celonis, Arctic AI, McKinsey analytics</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>15-25% EBITDA improvement identified</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Value Creation</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Pricing Optimization</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>ML-driven pricing recommendations for portfolio companies based on market dynamics</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Price Elasticity ML, Competitive Analysis</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Custom ML models, Anaplan, PROS</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>3-7% revenue increase</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Value Creation</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Customer Analytics</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Predictive models for customer churn, LTV, and acquisition optimization</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Classification ML, Cohort Analysis</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Amplitude, Mixpanel, custom models</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>20% reduction in churn</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Exit &amp; Valuation</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Comparable Company Analysis</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>AI-powered identification and analysis of comparable companies for valuation</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Similarity Matching, Financial Analysis</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>PitchBook, CapIQ, AlphaSense</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>50% faster comp selection</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Exit &amp; Valuation</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Exit Timing Optimization</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Predictive models suggesting optimal exit windows based on market conditions</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Time Series ML, Market Signals</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>PitchBook, custom models</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Improved exit multiples</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Exit &amp; Valuation</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Sell-side Preparation</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>AI-assisted creation of CIMs, management presentations from data room contents</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Document Generation, LLM</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Hebbia, DealRoom</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>40% faster preparation</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add AI Strategy Roadmaps tab with 23 downloadable PDFs
Added new 'AI Strategy Roadmaps' sheet containing free downloadable
AI strategy documents from major consulting and research firms:

Sources included:
- McKinsey (3): State of AI 2025, Agentic AI Advantage
- Deloitte (2): Tech Trends 2026, AI Governance Roadmap
- Accenture (5): Technology Vision 2025, Front-Runners Guide
- BCG (3): AI Radar 2026, Procurement AI
- KPMG (4): Intelligent Tech Enterprise, Customer Excellence
- PwC (1): AI Readiness
- EY (1): AI Regulatory Landscape
- WEF (4): Blueprint for Intelligent Economies, AI Sovereignty

All documents are:
- Free to download (no paywall)
- PDF format
- Longer than 5 pages
- Published 2024-2026

Also added Task 7 to daily automation for monthly roadmap monitoring
and Step 2d to the daily-ai-update skill.

https://claude.ai/code/session_01B5awo4mUbf5S6xgp9viyuG
</commit_message>
<xml_diff>
--- a/AI_Use_Cases_Comprehensive_2026.xlsx
+++ b/AI_Use_Cases_Comprehensive_2026.xlsx
@@ -21,6 +21,7 @@
     <sheet name="PE &amp; M&amp;A AI Use Cases" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Legal Tech AI Repos" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Manufacturing &amp; Distribution" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="AI Strategy Roadmaps" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +63,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="12">
@@ -178,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -236,6 +241,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -601,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -996,7 +1004,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="23" t="inlineStr">
         <is>
@@ -1076,9 +1083,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
@@ -5026,6 +5030,958 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Document Title</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Pages/Length</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>Download Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>McKinsey</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>The State of AI in 2025: Agents, Innovation, and Transformation</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>Comprehensive survey of 1,993 participants across 105 nations on AI adoption, value creation, and organizational rewiring</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>40+</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G2" s="25" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/~/media/mckinsey/business%20functions/quantumblack/our%20insights/the%20state%20of%20ai/november%202025/the-state-of-ai-2025-agents-innovation_cmyk-v1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>McKinsey</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>The State of AI: How Organizations Are Rewiring to Capture Value</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Analysis of how leading organizations transform operations using AI across business functions</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>30+</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G3" s="25" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/~/media/mckinsey/business%20functions/quantumblack/our%20insights/the%20state%20of%20ai/2025/the-state-of-ai-how-organizations-are-rewiring-to-capture-value_final.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>McKinsey</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Seizing the Agentic AI Advantage</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Strategic guide on deploying agentic AI for enterprise transformation. Only 1% of enterprises view gen AI strategies as mature</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>25+</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G4" s="25" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/~/media/mckinsey/business%20functions/quantumblack/our%20insights/seizing%20the%20agentic%20ai%20advantage/seizing-the-agentic-ai-advantage.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Tech Trends 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Annual technology trends report covering AI infrastructure, data bottlenecks, and enterprise AI adoption strategies</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>100+</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G5" s="25" t="inlineStr">
+        <is>
+          <t>https://mkto.deloitte.com/rs/712-CNF-326/images/DI_Tech-trends-2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>AI Board Governance Roadmap</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Framework for boards of directors to understand AI oversight roles with guiding questions for effective governance</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>20+</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G6" s="25" t="inlineStr">
+        <is>
+          <t>https://boardmember.com/wp-content/uploads/2025/07/AI-Governance-Roadmap.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Technology Vision 2025: AI - A Declaration of Autonomy</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>25th annual tech trends report exploring AI-powered autonomy and trust as key business challenges</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G7" s="25" t="inlineStr">
+        <is>
+          <t>https://www.accenture.com/content/dam/accenture/final/accenture-com/document-3/Accenture-Tech-Vision-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Reinvention in the Age of Generative AI</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Executive summary with projections through 2026 showing 15%+ revenue growth for AI reinvention leaders</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>20+</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G8" s="25" t="inlineStr">
+        <is>
+          <t>https://www.accenture.com/content/dam/accenture/final/accenture-com/document-2/Accenture-reinvention-in-the-age-of-generative-AI-executive-summary.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>The Front-Runners' Guide to Scaling AI</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Lessons from industry leaders on using agentic AI for efficiency and strategic reinvention</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>30+</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G9" s="25" t="inlineStr">
+        <is>
+          <t>https://www.accenture.com/content/dam/accenture/final/accenture-com/document-3/Accenture-Front-Runners-Guide-Scaling-AI-2025-POV.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>AI: Built to Scale</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Study on AI-enabled business strategy, top characteristics for scaling AI, and financial results</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>40+</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G10" s="25" t="inlineStr">
+        <is>
+          <t>https://www.accenture.com/content/dam/accenture/final/a-com-migration/thought-leadership-assets/accenture-built-to-scale-pdf-report.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Accenture</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>AI Roadmap: The Journey to Live (Infographic)</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Visual roadmap covering AI implementation checkpoints and adjustments</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>10+</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G11" s="25" t="inlineStr">
+        <is>
+          <t>https://www.accenture.com/content/dam/accenture/final/a-com-migration/pdf/pdf-122/accenture-ai-roadmap-journey-to-live-infographic.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>BCG</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>AI Radar 2026: As AI Investments Surge, CEOs Take the Lead</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Survey of 2,360 executives on agentic AI, CEO leadership in AI, and organizational transformation</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>30+</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G12" s="25" t="inlineStr">
+        <is>
+          <t>https://web-assets.bcg.com/73/8e/cc44cbc14a3b81695f8a3de28ff1/ai-radar-2026-web-jan-2026-edit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>BCG</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Future of Procurement with AI 2025</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>AI opportunities for strategic advantages and operational efficiencies with up to 15% savings potential</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>20+</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G13" s="25" t="inlineStr">
+        <is>
+          <t>https://media-publications.bcg.com/BCG-Executive-Perspectives-Future-of-Procurement-with-AI-2025-27Feb2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>BCG</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Driving Sustainable Cost Advantage with AI</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>90% of executives planning AI investments for cost reduction over next 18 months</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>15+</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G14" s="25" t="inlineStr">
+        <is>
+          <t>https://media-publications.bcg.com/BCG-Executive-Perspectives-Driving-Sustainable-Cost-Adv-with-AI-EP15-20May2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>KPMG</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Intelligent Tech Enterprise: A Blueprint for AI-Driven Transformation</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>AI strategy framework covering responsible executive appointment, use case identification, and regulatory alignment</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>25+</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G15" s="25" t="inlineStr">
+        <is>
+          <t>https://assets.kpmg.com/content/dam/kpmg/ng/pdf/2025/intelligent-industries/Intelligent%20tech%20-%20Report.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>KPMG</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Global Customer Experience Excellence 2025-2026</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Redefining excellence in the age of agentic AI - covers AI capable of sensing, reasoning, and acting</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G16" s="25" t="inlineStr">
+        <is>
+          <t>https://assets.kpmg.com/content/dam/kpmgsites/xx/pdf/2025/10/global-customer-experience-excellence-2025-2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>KPMG</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>AI Workforce: From Hype to Hard Truths</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>What it takes to deliver AI value - practical guidance on AI workforce transformation</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>20+</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G17" s="25" t="inlineStr">
+        <is>
+          <t>https://assets.kpmg.com/content/dam/kpmgsites/se/pdf/2025/ai-workforce-from-hype-to-hard-truths.pdf.coredownload.inline.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>KPMG</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>AI in Retail Report</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Practical examples of AI in retail with insights from Global Tech Report and CEO Outlook</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>30+</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G18" s="25" t="inlineStr">
+        <is>
+          <t>https://assets.kpmg.com/content/dam/kpmgsites/xx/pdf/2026/01/ai-in-retail-report.pdf.coredownload.inline.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>AI Readiness: Shaping the Future AI Landscape</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>National AI capabilities assessment across semiconductors, infrastructure, models, and services</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>40+</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G19" s="25" t="inlineStr">
+        <is>
+          <t>https://www.pwc.com/gx/en/industries/technology/ai-readiness.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>AI Global Regulatory Landscape</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Comprehensive overview of global AI regulations and governance frameworks</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>30+</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G20" s="25" t="inlineStr">
+        <is>
+          <t>https://www.ey.com/content/dam/ey-unified-site/ey-com/en-gl/insights/ai/documents/ey-the-artificial-intelligence-ai-global-regulatory-landscape-final.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="50" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>WEF</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Blueprint for Intelligent Economies</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Guidance for nations to achieve successful AI revolution regardless of digital maturity level</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>40+</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G21" s="25" t="inlineStr">
+        <is>
+          <t>https://reports.weforum.org/docs/WEF_A_Blueprint_for_Intelligent_Economies_2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="50" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>WEF</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Rethinking AI Sovereignty: Pathways to Competitiveness</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Policy guidance for enabling AI-driven economy through partnership over ownership</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>35+</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G22" s="25" t="inlineStr">
+        <is>
+          <t>https://www3.weforum.org/docs/WEF_Rethinking_AI_Sovereignty_Pathways_to_Competitiveness_through_Strategic_Investments_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="50" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>WEF</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Four Futures for Jobs: AI and Talent in 2030</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Scenario analysis for future of jobs at intersection of AI advancement and workforce readiness</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>30+</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G23" s="25" t="inlineStr">
+        <is>
+          <t>https://reports.weforum.org/docs/WEF_Four_Futures_for_Jobs_in_the_New_Economy_AI_and_Talent_in_2030_2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="50" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>WEF</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>AI in Action: Beyond Experimentation to Transform Industry</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Comprehensive roadmap for businesses and governments to adopt and scale AI</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G24" s="25" t="inlineStr">
+        <is>
+          <t>https://reports.weforum.org/docs/WEF_AI_in_Action_Beyond_Experimentation_to_Transform_Industry_2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Total Documents:</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sources:</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>McKinsey (3), Deloitte (2), Accenture (5), BCG (3), KPMG (4), PwC (1), EY (1), WEF (4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>All links verified:</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Free PDF downloads, no paywall</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add 8 additional AI Strategy Roadmaps (31 total)
Added resources from user-specified sources:
- C3.ai: Enterprise AI Roadmap, Buyer's Guide (use case qualification)
- WEF: AI C-Suite Toolkit (governance & risk framing)
- Info-Tech: Build Your AI Strategy Roadmap (maturity/prioritization tools)
- RTS Labs: Enterprise AI Roadmap (12-18 month phased plan)
- 3Cloud: AI Strategy Roadmap eBook
- Microsoft: AI Strategy Roadmap
- Applied AI: Elements of Comprehensive AI Strategy

Updated automation sources table with 12 firms (was 8).
Total downloadable documents: 31

https://claude.ai/code/session_01B5awo4mUbf5S6xgp9viyuG
</commit_message>
<xml_diff>
--- a/AI_Use_Cases_Comprehensive_2026.xlsx
+++ b/AI_Use_Cases_Comprehensive_2026.xlsx
@@ -183,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -242,6 +242,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5036,7 +5039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5936,44 +5939,341 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>C3.ai</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Best Practices in Developing an Enterprise AI Roadmap</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Use case qualification model with guidance on determining business value and feasibility. Includes prioritization and sequencing framework.</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>15-17</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="G26" s="25" t="inlineStr">
+        <is>
+          <t>https://c3.ai/wp-content/uploads/2020/06/Best-Practices-in-Developing-an-Enterprise-AI-Roadmap.pdf</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
-      <c r="A27" s="23" t="inlineStr">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>C3.ai</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Enterprise AI Buyer's Guide</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Enterprise AI Requirements Checklist specifying all capabilities an AI platform must provide for complete, robust solutions</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>20+</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="G27" s="25" t="inlineStr">
+        <is>
+          <t>https://c3.ai/wp-content/uploads/2020/06/Enterprise-AI-Buyers-Guide.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>WEF</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Empowering AI Leadership: AI C-Suite Toolkit</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Comprehensive toolkit for C-suite executives covering AI strategy, governance, risk management, and responsible AI implementation</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="G28" s="25" t="inlineStr">
+        <is>
+          <t>https://www3.weforum.org/docs/WEF_Empowering_AI_Leadership_2022.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>3Cloud</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>AI Strategy Roadmap eBook</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Practical guidance for AI implementation covering readiness assessment and path to successful deployment</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>25+</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G29" s="25" t="inlineStr">
+        <is>
+          <t>https://3cloudsolutions.com/wp-content/uploads/2025/10/AI-Strategy-Roadmap-eBook.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>The AI Strategy Roadmap</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Insights from IT leaders and business decision makers on successfully integrating AI and realizing business value</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>30+</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G30" s="25" t="inlineStr">
+        <is>
+          <t>https://replyfabric.ai/documents/microsoft-the-ai-strategy-roadmap-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Info-Tech</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Build Your AI Strategy Roadmap Blueprint</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>4-step framework with AI Maturity Assessment Tool and Prioritization/Roadmap Planning frameworks. Includes governance principles.</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Multi-page</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>Web + Tools</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G31" s="25" t="inlineStr">
+        <is>
+          <t>https://www.infotech.com/research/build-your-ai-strategy-roadmap-storyboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>RTS Labs</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Enterprise AI Roadmap: Complete 2026 Guide</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>12-18 month phased plan combining strategy + engineering + MLOps. Business-first lens mapping AI to financial outcomes.</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Long article</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G32" s="25" t="inlineStr">
+        <is>
+          <t>https://rtslabs.com/enterprise-ai-roadmap/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Applied AI</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Elements of a Comprehensive AI Strategy</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Framework covering AI strategy components for enterprise implementation</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>15+</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G33" s="25" t="inlineStr">
+        <is>
+          <t>https://aai.frb.io/assets/videos/AppliedAI_Elements-of-a-comprehensive-AI-Strategy.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Total Documents:</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="B37" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Sources:</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>McKinsey (3), Deloitte (2), Accenture (5), BCG (3), KPMG (4), PwC (1), EY (1), WEF (4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>McKinsey (3), Deloitte (2), Accenture (5), BCG (3), KPMG (4), PwC (1), EY (1), WEF (5), C3.ai (2), 3Cloud (1), Microsoft (1), Info-Tech (1), RTS Labs (1), Applied AI (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>All links verified:</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Free PDF downloads, no paywall</t>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Free PDF/Web downloads, no paywall (except Info-Tech tools may require contact)</t>
         </is>
       </c>
     </row>

</xml_diff>